<commit_message>
give chart titles their own space
</commit_message>
<xml_diff>
--- a/public/sales-report-template.xlsx
+++ b/public/sales-report-template.xlsx
@@ -349,6 +349,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -545,6 +546,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -724,6 +726,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -882,6 +885,7 @@
           </a:p>
         </txPr>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -920,6 +924,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1078,6 +1083,7 @@
           </a:p>
         </txPr>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -1116,6 +1122,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -1295,6 +1302,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1453,6 +1461,7 @@
           </a:p>
         </txPr>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -1491,6 +1500,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1649,6 +1659,7 @@
           </a:p>
         </txPr>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -1687,6 +1698,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1883,6 +1895,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -2062,6 +2075,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -2220,6 +2234,7 @@
           </a:p>
         </txPr>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -2258,6 +2273,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -2416,6 +2432,7 @@
           </a:p>
         </txPr>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -2454,6 +2471,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>

</xml_diff>